<commit_message>
Add SOH report for 2026-10-17
</commit_message>
<xml_diff>
--- a/reports/SOH_16_10_2026.xlsx
+++ b/reports/SOH_16_10_2026.xlsx
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>12758</v>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>10261</v>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>538</v>
+        <v>526</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>8319</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1006</v>
+        <v>997</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>10500</v>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>555</v>
+        <v>549</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>24000</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>959</v>
+        <v>953</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1166</v>
+        <v>1160</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="D60" s="2" t="n">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>26500</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>508</v>
+        <v>502</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>26500</v>
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D68" s="2" t="n">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>26500</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>525</v>
+        <v>513</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>2506</v>
+        <v>2494</v>
       </c>
       <c r="E110" s="3" t="n">
         <v>3500</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2055</v>
+        <v>2043</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="D128" s="2" t="n">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="E128" s="3" t="n">
         <v>3500</v>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E135" s="3" t="n">
         <v>2500</v>
@@ -4685,7 +4685,7 @@
         </is>
       </c>
       <c r="D152" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E152" s="3" t="n">
         <v>8833</v>
@@ -5313,7 +5313,7 @@
         </is>
       </c>
       <c r="D175" s="2" t="n">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="E175" s="3" t="n">
         <v>13500</v>
@@ -7441,7 +7441,7 @@
         </is>
       </c>
       <c r="D254" s="2" t="n">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E254" s="3" t="n">
         <v>8367</v>
@@ -7469,7 +7469,7 @@
         </is>
       </c>
       <c r="D255" s="2" t="n">
-        <v>836</v>
+        <v>824</v>
       </c>
       <c r="E255" s="3" t="n">
         <v>11491</v>
@@ -8421,7 +8421,7 @@
         </is>
       </c>
       <c r="D289" s="2" t="n">
-        <v>1258</v>
+        <v>1246</v>
       </c>
       <c r="E289" s="3" t="n">
         <v>7347</v>
@@ -9037,7 +9037,7 @@
         </is>
       </c>
       <c r="D311" s="2" t="n">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E311" s="3" t="n">
         <v>12300</v>
@@ -9065,7 +9065,7 @@
         </is>
       </c>
       <c r="D312" s="2" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E312" s="3" t="n">
         <v>26979</v>
@@ -9513,7 +9513,7 @@
         </is>
       </c>
       <c r="D328" s="2" t="n">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="E328" s="3" t="n">
         <v>12666</v>
@@ -9850,7 +9850,7 @@
         </is>
       </c>
       <c r="D340" s="2" t="n">
-        <v>118</v>
+        <v>-122</v>
       </c>
       <c r="E340" s="3" t="n">
         <v>2500</v>
@@ -9962,7 +9962,7 @@
         </is>
       </c>
       <c r="D344" s="2" t="n">
-        <v>1236</v>
+        <v>1230</v>
       </c>
       <c r="E344" s="3" t="n">
         <v>10170</v>
@@ -11390,7 +11390,7 @@
         </is>
       </c>
       <c r="D395" s="2" t="n">
-        <v>1518</v>
+        <v>1512</v>
       </c>
       <c r="E395" s="3" t="n">
         <v>13752</v>
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="D400" s="2" t="n">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E400" s="3" t="n">
         <v>13511</v>
@@ -11586,7 +11586,7 @@
         </is>
       </c>
       <c r="D402" s="2" t="n">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="E402" s="3" t="n">
         <v>9765</v>
@@ -11754,7 +11754,7 @@
         </is>
       </c>
       <c r="D408" s="2" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="E408" s="3" t="n">
         <v>11443</v>
@@ -12622,7 +12622,7 @@
         </is>
       </c>
       <c r="D439" s="2" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E439" s="3" t="n">
         <v>14565</v>
@@ -13070,7 +13070,7 @@
         </is>
       </c>
       <c r="D455" s="2" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E455" s="3" t="n">
         <v>8734</v>
@@ -13154,7 +13154,7 @@
         </is>
       </c>
       <c r="D458" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E458" s="3" t="n">
         <v>8856</v>
@@ -14050,7 +14050,7 @@
         </is>
       </c>
       <c r="D490" s="2" t="n">
-        <v>1773</v>
+        <v>1767</v>
       </c>
       <c r="E490" s="3" t="n">
         <v>15262</v>
@@ -14246,7 +14246,7 @@
         </is>
       </c>
       <c r="D497" s="2" t="n">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E497" s="3" t="n">
         <v>23611</v>
@@ -14834,7 +14834,7 @@
         </is>
       </c>
       <c r="D518" s="2" t="n">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E518" s="3" t="n">
         <v>12504</v>
@@ -15338,7 +15338,7 @@
         </is>
       </c>
       <c r="D536" s="2" t="n">
-        <v>5038</v>
+        <v>5032</v>
       </c>
       <c r="E536" s="3" t="n">
         <v>10621</v>
@@ -15478,7 +15478,7 @@
         </is>
       </c>
       <c r="D541" s="2" t="n">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="E541" s="3" t="n">
         <v>22302</v>
@@ -15534,7 +15534,7 @@
         </is>
       </c>
       <c r="D543" s="2" t="n">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="E543" s="3" t="n">
         <v>12816</v>
@@ -16094,7 +16094,7 @@
         </is>
       </c>
       <c r="D563" s="2" t="n">
-        <v>372</v>
+        <v>351</v>
       </c>
       <c r="E563" s="3" t="n">
         <v>13522</v>
@@ -17018,7 +17018,7 @@
         </is>
       </c>
       <c r="D596" s="2" t="n">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="E596" s="3" t="n">
         <v>9563</v>
@@ -17354,7 +17354,7 @@
         </is>
       </c>
       <c r="D608" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E608" s="3" t="n">
         <v>13111</v>
@@ -17634,7 +17634,7 @@
         </is>
       </c>
       <c r="D618" s="2" t="n">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="E618" s="3" t="n">
         <v>8331</v>
@@ -17943,7 +17943,7 @@
         </is>
       </c>
       <c r="D629" s="2" t="n">
-        <v>3761</v>
+        <v>3755</v>
       </c>
       <c r="E629" s="3" t="n">
         <v>10251</v>
@@ -17999,7 +17999,7 @@
         </is>
       </c>
       <c r="D631" s="2" t="n">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="E631" s="3" t="n">
         <v>9776</v>
@@ -18111,7 +18111,7 @@
         </is>
       </c>
       <c r="D635" s="2" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E635" s="3" t="n">
         <v>8559</v>
@@ -18167,7 +18167,7 @@
         </is>
       </c>
       <c r="D637" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E637" s="3" t="n">
         <v>12330</v>
@@ -19651,7 +19651,7 @@
         </is>
       </c>
       <c r="D690" s="2" t="n">
-        <v>259</v>
+        <v>244</v>
       </c>
       <c r="E690" s="3" t="n">
         <v>9444</v>
@@ -21779,7 +21779,7 @@
         </is>
       </c>
       <c r="D766" s="2" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E766" s="3" t="n">
         <v>20702</v>
@@ -21947,7 +21947,7 @@
         </is>
       </c>
       <c r="D772" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E772" s="3" t="n">
         <v>10710</v>
@@ -22983,7 +22983,7 @@
         </is>
       </c>
       <c r="D809" s="2" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E809" s="3" t="n">
         <v>17617</v>
@@ -23459,7 +23459,7 @@
         </is>
       </c>
       <c r="D826" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E826" s="3" t="n">
         <v>9499</v>
@@ -24579,7 +24579,7 @@
         </is>
       </c>
       <c r="D866" s="2" t="n">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="E866" s="3" t="n">
         <v>7564</v>
@@ -24635,7 +24635,7 @@
         </is>
       </c>
       <c r="D868" s="2" t="n">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="E868" s="3" t="n">
         <v>16983</v>
@@ -25056,7 +25056,7 @@
         </is>
       </c>
       <c r="D883" s="2" t="n">
-        <v>-24</v>
+        <v>-36</v>
       </c>
       <c r="E883" s="3" t="n">
         <v>6718</v>
@@ -30016,7 +30016,7 @@
         </is>
       </c>
       <c r="D1060" s="2" t="n">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="E1060" s="3" t="n">
         <v>5517</v>
@@ -30324,7 +30324,7 @@
         </is>
       </c>
       <c r="D1071" s="2" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E1071" s="3" t="n">
         <v>11795</v>
@@ -30744,7 +30744,7 @@
         </is>
       </c>
       <c r="D1086" s="2" t="n">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="E1086" s="3" t="n">
         <v>14904</v>
@@ -30828,7 +30828,7 @@
         </is>
       </c>
       <c r="D1089" s="2" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E1089" s="3" t="n">
         <v>11970</v>
@@ -31305,7 +31305,7 @@
         </is>
       </c>
       <c r="D1106" s="2" t="n">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="E1106" s="3" t="n">
         <v>10480</v>
@@ -31417,7 +31417,7 @@
         </is>
       </c>
       <c r="D1110" s="2" t="n">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E1110" s="3" t="n">
         <v>7008</v>
@@ -32509,7 +32509,7 @@
         </is>
       </c>
       <c r="D1149" s="2" t="n">
-        <v>644</v>
+        <v>636</v>
       </c>
       <c r="E1149" s="3" t="n">
         <v>12935</v>
@@ -34385,7 +34385,7 @@
         </is>
       </c>
       <c r="D1216" s="2" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="E1216" s="3" t="n">
         <v>14752</v>
@@ -34525,7 +34525,7 @@
         </is>
       </c>
       <c r="D1221" s="2" t="n">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="E1221" s="3" t="n">
         <v>8325</v>
@@ -34581,7 +34581,7 @@
         </is>
       </c>
       <c r="D1223" s="2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E1223" s="3" t="n">
         <v>8155</v>
@@ -38249,7 +38249,7 @@
         </is>
       </c>
       <c r="D1354" s="2" t="n">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E1354" s="3" t="n">
         <v>14320</v>
@@ -39593,7 +39593,7 @@
         </is>
       </c>
       <c r="D1402" s="2" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E1402" s="3" t="n">
         <v>7139</v>
@@ -39649,7 +39649,7 @@
         </is>
       </c>
       <c r="D1404" s="2" t="n">
-        <v>685</v>
+        <v>679</v>
       </c>
       <c r="E1404" s="3" t="n">
         <v>12595</v>
@@ -39677,7 +39677,7 @@
         </is>
       </c>
       <c r="D1405" s="2" t="n">
-        <v>1444</v>
+        <v>1438</v>
       </c>
       <c r="E1405" s="3" t="n">
         <v>10295</v>
@@ -42113,7 +42113,7 @@
         </is>
       </c>
       <c r="D1492" s="2" t="n">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E1492" s="3" t="n">
         <v>15697</v>
@@ -42141,7 +42141,7 @@
         </is>
       </c>
       <c r="D1493" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E1493" s="3" t="n">
         <v>15302</v>
@@ -42253,7 +42253,7 @@
         </is>
       </c>
       <c r="D1497" s="2" t="n">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="E1497" s="3" t="n">
         <v>8626</v>
@@ -43065,7 +43065,7 @@
         </is>
       </c>
       <c r="D1526" s="2" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E1526" s="3" t="n">
         <v>16643</v>
@@ -43429,7 +43429,7 @@
         </is>
       </c>
       <c r="D1539" s="2" t="n">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="E1539" s="3" t="n">
         <v>12419</v>
@@ -43541,7 +43541,7 @@
         </is>
       </c>
       <c r="D1543" s="2" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E1543" s="3" t="n">
         <v>14050</v>
@@ -44073,7 +44073,7 @@
         </is>
       </c>
       <c r="D1562" s="2" t="n">
-        <v>2494</v>
+        <v>2470</v>
       </c>
       <c r="E1562" s="3" t="n">
         <v>7312</v>
@@ -44101,7 +44101,7 @@
         </is>
       </c>
       <c r="D1563" s="2" t="n">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="E1563" s="3" t="n">
         <v>9332</v>
@@ -44129,7 +44129,7 @@
         </is>
       </c>
       <c r="D1564" s="2" t="n">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="E1564" s="3" t="n">
         <v>10267</v>
@@ -44157,7 +44157,7 @@
         </is>
       </c>
       <c r="D1565" s="2" t="n">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E1565" s="3" t="n">
         <v>16495</v>
@@ -44241,7 +44241,7 @@
         </is>
       </c>
       <c r="D1568" s="2" t="n">
-        <v>142</v>
+        <v>118</v>
       </c>
       <c r="E1568" s="3" t="n">
         <v>7390</v>
@@ -44381,7 +44381,7 @@
         </is>
       </c>
       <c r="D1573" s="2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E1573" s="3" t="n">
         <v>7304</v>

</xml_diff>